<commit_message>
Update employee import template and logic
- Updated employee_template.xlsx to include first_name and last_name as required fields.
- Made full_name optional in the template.
- Updated modules/import/index.php documentation to reflect these changes.
- Updated itm_handle_json_table_import in config/config.php to prioritize explicit first_name and last_name fields over full_name splitting.

Co-authored-by: google-labs-jules[bot] <161369871+google-labs-jules[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/modules/import/employee_template.xlsx
+++ b/modules/import/employee_template.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +28,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FF0000"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
     </font>
   </fonts>
   <fills count="3">
@@ -56,10 +59,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,36 +430,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>first_name</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>last_name</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>full_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>username</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>job_title</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>employee_id</t>
         </is>
@@ -463,30 +478,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>John</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Smith</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>John Smith</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>john@example.com</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>jsmith</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>+123456789</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>EMP001</t>
         </is>

</xml_diff>

<commit_message>
Update Employee import fields and Excel template
- Added support for emergency contact details and birthday in employee import.
- Explicitly excluded sensitive fields (password, roles, access levels) from import logic for security.
- Updated documentation and generated Excel template with all supported fields and UK date format examples.

Co-authored-by: google-labs-jules[bot] <161369871+google-labs-jules[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/modules/import/employee_template.xlsx
+++ b/modules/import/employee_template.xlsx
@@ -30,21 +30,15 @@
       <color rgb="00FF0000"/>
     </font>
     <font>
-      <color rgb="00000000"/>
+      <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D4EDDA"/>
-        <bgColor rgb="00D4EDDA"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -59,12 +53,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,48 +422,154 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:X2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="27" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="17" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="24" max="24"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>first_name</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>last_name</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>full_name</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>username</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>phone</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>job_title</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>employee_id</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Display Name</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Full Name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Work Email</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Personal Email</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Emergency Contact Name</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Emergency Contact Relationship</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Emergency Contact Phone</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Mobile Phone</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>External Number</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Dect</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Extension</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Employee Code</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>External ID</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Insurance N</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Username</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>Job Code</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>Request Date</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>Requested By</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
@@ -488,32 +586,112 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>John S.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>John Smith</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>john@example.com</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>john@company.com</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>john.personal@gmail.com</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Jane Smith</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Spouse</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>+1234567891</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>+1234567890</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>+1987654321</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>5678</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>EMP001</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>EXT-999</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>INS-12345</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>jsmith</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>+123456789</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Software Engineer</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EMP001</t>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>JOB-101</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Key member of IT.</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>31/01/2026</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>01/02/2026</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>15/05/1990</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>

</xml_diff>